<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.002-05 Nina souffle et fait une pause
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-05.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-05.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Les cubes bleus de Nino</t>
+          <t>Nina souffle et fait une pause</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chambre</t>
+          <t>chambre, lit, bois, barre, pied du lit, cubes, coton, rayon, point de lumière</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, papa, maman</t>
+          <t>Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut une petite tour bleue. Les cubes tombent. Il souffle, fait une pause, puis reprend un cube.</t>
+          <t>Un rayon tiède dort sur le bois. Sur le pied du lit, un éclat de lit luit. Nina veut empiler, maintenant. Cubes tombent, poitrine trop vite, sourire parti. Maman s'accroupit. Elle souffle. Pause. Merci vécu. Les cubes glissent sur le coton du lit. Elle refuse d'empiler, souffle, pause. Un éclat de lit tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, la maison est douce. Le rideau jaune bouge un peu. Il frotte la fenêtre, tout léger. Le doudou attend sur l'oreiller. Un oiseau chante, dehors. Le couloir sent le savon. La sieste est finie, Nino. J'ouvre un peu le rideau. Un rayon arrive sur le tapis. Le rayon est chaud. Le tapis brille, maman. Oui. Il est doux aussi. Tes cubes sont près du lit. On peut jouer, tout calme. En ce moment, Nino joue. Il est dans sa chambre. Les cubes sont bleus. Nino veut une petite tour. Une tour, maman. Tu poses un cube, tout doux ? Nino pose un cube. Puis un autre. Ça fait un petit bruit. La tour tremble. Les cubes tombent. Ça fait un bruit sec. Nino sent sa poitrine aller vite. Son ventre se serre. C'est trop. Je suis fâché. La tour est tombée. Tu es fâché. On peut souffler. On peut faire une pause. Nino s'assoit sur le tapis. Il pose les mains sur ses genoux. Nino souffle comme le vent. Une fois. Deux fois. Il fait une pause. La chambre redevient calme. Je souffle. Je fais une pause. Bravo, Nino. C'est calme. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Tout doucement. Nino reprend un cube bleu. Il construit tout doucement. La tour est petite. Elle tient.</t>
+          <t>Un rayon tiède dort sur le bois. Il est chaud, papa. Tu le vois, le rayon ? Oui, papa. Ça sent le coton, un peu sec. Tu le sens, le coton ? Oui, maman. Une barre du lit tinte. Elle sonne, maman. Le lit est là, sous le rayon. Je le vois. Papa tapote le pied du lit. Toc, toc, sur le bois. Tu entends le bois, Nina ? Oui, il sonne. Maman pose la main près du bois. Le bois est lisse, un peu tiède. Sur le bois, un éclat de lit luit. Il luit, papa. Tu le vois, sur le bois ? Oui, un petit point. La lumière le touche. Un rayon glisse le long du lit. Nina connaît cette chambre. Le point est nouveau. Tu t'assois près du lit ? Un peu. Un cube bleu brille près du bois. Il est bleu. Les cubes sont là, tu vois ? Oui, papa. En ce moment, Nina prend un cube. Je veux empiler, maintenant ! Tout de suite ? Oui, papa. Le cube est lisse, un peu froid. Tu poses un cube ? Oui, maman. Nina pose un cube trop vite. Puis un autre, trop haut. La pile penche. Elle monte ! Les cubes tombent. Ça fait un bruit sec. Oh. Le sourire de Nina disparaît. Dans sa poitrine, ça va trop vite. L'envie et la peur se heurtent. Ses épaules montent un peu. Maman s'accroupit à la même hauteur. Tu vois les cubes, Nina ? Oui, maman. Ta poitrine va vite, Nina ? Un peu, papa. C'est trop. Nina souffle vers ses mains. Fouu. Elle fait une pause, près du lit. L'éclat de lit tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, la maison est douce. Le rideau jaune bouge un peu. Il frotte la fenêtre, tout léger. Le doudou attend sur l'oreiller. Un oiseau chante, dehors. Le couloir sent le savon. La sieste est finie, Nino. J'ouvre un peu le rideau. Un rayon arrive sur le tapis. Le rayon est chaud. Le tapis brille, maman. Oui. Il est doux aussi. Tes cubes sont près du lit. On peut jouer, tout calme. En ce moment, Nino joue. Il est dans sa chambre. Les cubes sont bleus. Nino veut une petite tour. Une tour, maman. Tu poses un cube, tout doux ? Nino pose un cube. Puis un autre. Ça fait un petit bruit. La tour tremble. Les cubes tombent. Ça fait un bruit sec. Nino sent sa poitrine aller vite. Son ventre se serre. C'est trop. Je suis fâché. La tour est tombée. Tu es fâché. On peut souffler. On peut faire une pause. Nino s'assoit sur le tapis. Il pose les mains sur ses genoux. Nino souffle comme le vent. Une fois. Deux fois. Il fait une pause. La chambre redevient calme. Je souffle. Je fais une pause. Bravo, Nino. C'est calme. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Tout doucement. Nino reprend un cube bleu. Il construit tout doucement. La tour est petite. Elle tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon tiède dort sur le bois. Il est chaud, papa. Tu le vois, le rayon ? Oui, papa. Ça sent le coton, un peu sec. Tu le sens, le coton ? Oui, maman. Une barre du lit tinte. Elle sonne, maman. Le lit est là, sous le rayon. Je le vois. Papa tapote le pied du lit. Toc, toc, sur le bois. Tu entends le bois, Nina ? Oui, il sonne. Maman pose la main près du bois. Le bois est lisse, un peu tiède. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de lit&lt;/emphasis&gt; luit. Il luit, papa. Tu le vois, sur le bois ? Oui, un petit point. La lumière le touche. Un rayon glisse le long du lit. Nina connaît cette chambre. Le point est nouveau. Tu t'assois près du lit ? Un peu. Un cube bleu brille près du bois. Il est bleu. Les cubes sont là, tu vois ? Oui, papa. En ce moment, Nina prend un cube. Je veux empiler, maintenant ! Tout de suite ? Oui, papa. Le cube est lisse, un peu froid. Tu poses un cube ? Oui, maman. Nina pose un cube trop vite. Puis un autre, trop haut. La pile penche. Elle monte ! Les cubes tombent. Ça fait un bruit sec. Oh. Le sourire de Nina disparaît. Dans sa poitrine, ça va trop vite. L'envie et la peur se heurtent. Ses épaules montent un peu. Maman s'accroupit à la même hauteur. Tu vois les cubes, Nina ? Oui, maman. Ta poitrine va vite, Nina ? Un peu, papa. C'est trop. Nina souffle vers ses mains. Fouu. Elle fait une pause, près du lit. L'éclat de lit tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Gaëlle joue dans sa chambre. Les cubes tombent. Ça fait un bruit sec. Gaëlle sent sa poitrine aller vite. Elle dit : c'est trop. Maman est près du lit. Maman dit : on peut &lt;emphasis&gt;souffler&lt;/emphasis&gt;. Gaëlle souffle comme le vent. Une fois. Deux fois. Elle s'assoit sur le tapis. Elle fait une pause. Ses mains se posent sur ses genoux. La chambre redevient calme. Gaëlle reprend un cube bleu. Elle construit tout doucement. Maman reste près d'elle. Souffler, puis une pause. On peut reprendre.&lt;/slow&gt; [pause]</t>
+          <t>Un rayon tiède dort sur le bois. Il est chaud, papa. Tu le vois, le rayon ? Oui, papa. Ça sent le coton, un peu sec. Tu le sens, le coton ? Oui, maman. Une barre du lit tinte. Elle sonne, maman. Le lit est là, sous le rayon. Je le vois. Papa tapote le pied du lit. Toc, toc, sur le bois. Tu entends le bois, Nina ? Oui, il sonne. Maman pose la main près du bois. Le bois est lisse, un peu tiède. Sur le bois, un &lt;emphasis&gt;éclat de lit&lt;/emphasis&gt; luit. Il luit, papa. Tu le vois, sur le bois ? Oui, un petit point. La lumière le touche. Un rayon glisse le long du lit. Nina connaît cette chambre. Le point est nouveau. Tu t'assois près du lit ? Un peu. Un cube bleu brille près du bois. Il est bleu. Les cubes sont là, tu vois ? Oui, papa. En ce moment, Nina prend un cube. Je veux empiler, maintenant ! Tout de suite ? Oui, papa. Le cube est lisse, un peu froid. Tu poses un cube ? Oui, maman. Nina pose un cube trop vite. Puis un autre, trop haut. La pile penche. Elle monte ! Les cubes tombent. Ça fait un bruit sec. Oh. Le sourire de Nina disparaît. Dans sa poitrine, ça va trop vite. L'envie et la peur se heurtent. Ses épaules montent un peu. Maman s'accroupit à la même hauteur. Tu vois les cubes, Nina ? Oui, maman. Ta poitrine va vite, Nina ? Un peu, papa. C'est trop. Nina souffle vers ses mains. Fouu. Elle fait une pause, près du lit. L'éclat de lit tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>souffler</t>
+          <t>éclat de lit</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,63 +1319,79 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=elle_veut_empiler_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Après la sieste, la maison est douce.
-narrateur|Le rideau jaune bouge un peu.
-narrateur|Il frotte la fenêtre, tout léger.
-narrateur|Le doudou attend sur l'oreiller.
-narrateur|Un oiseau chante, dehors.
-narrateur|Le couloir sent le savon.
-maman|La sieste est finie, Nino.
-papa|J'ouvre un peu le rideau.
-narrateur|Un rayon arrive sur le tapis.
-narrateur|Le rayon est chaud.
-enfant-m|Le tapis brille, maman.
-maman|Oui. Il est doux aussi.
-papa|Tes cubes sont près du lit.
-maman|On peut jouer, tout calme.
-narrateur|En ce moment, Nino joue.
-narrateur|Il est dans sa chambre.
-narrateur|Les cubes sont bleus.
-narrateur|Nino veut une petite tour.
-enfant-m|Une tour, maman.
-maman|Tu poses un cube, tout doux ?
-narrateur|Nino pose un cube.
-narrateur|Puis un autre.
-narrateur|Ça fait un petit bruit.
-narrateur|La tour tremble.
+          <t>narrateur|Un rayon tiède dort sur le bois.
+enfant-f|Il est chaud, papa.
+papa|Tu le vois, le rayon ?
+enfant-f|Oui, papa.
+narrateur|Ça sent le coton, un peu sec.
+maman|Tu le sens, le coton ?
+enfant-f|Oui, maman.
+narrateur|Une barre du lit tinte.
+enfant-f|Elle sonne, maman.
+maman|Le lit est là, sous le rayon.
+enfant-f|Je le vois.
+narrateur|Papa tapote le pied du lit.
+narrateur|Toc, toc, sur le bois.
+papa|Tu entends le bois, Nina ?
+enfant-f|Oui, il sonne.
+narrateur|Maman pose la main près du bois.
+narrateur|Le bois est lisse, un peu tiède.
+narrateur|Sur le bois, un éclat de lit luit.
+enfant-f|Il luit, papa.
+papa|Tu le vois, sur le bois ?
+enfant-f|Oui, un petit point.
+maman|La lumière le touche.
+narrateur|Un rayon glisse le long du lit.
+narrateur|Nina connaît cette chambre.
+enfant-f|Le point est nouveau.
+maman|Tu t'assois près du lit ?
+enfant-f|Un peu.
+narrateur|Un cube bleu brille près du bois.
+enfant-f|Il est bleu.
+papa|Les cubes sont là, tu vois ?
+enfant-f|Oui, papa.
+narrateur|En ce moment, Nina prend un cube.
+enfant-f|Je veux empiler, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Le cube est lisse, un peu froid.
+maman|Tu poses un cube ?
+enfant-f|Oui, maman.
+narrateur|Nina pose un cube trop vite.
+narrateur|Puis un autre, trop haut.
+narrateur|La pile penche.
+enfant-f|Elle monte !
 narrateur|Les cubes tombent.
 narrateur|Ça fait un bruit sec.
-narrateur|Nino sent sa poitrine aller vite.
-narrateur|Son ventre se serre.
-enfant-m|C'est trop. Je suis fâché.
-maman|La tour est tombée. Tu es fâché.
-maman|On peut souffler.
-papa|On peut faire une pause.
-narrateur|Nino s'assoit sur le tapis.
-narrateur|Il pose les mains sur ses genoux.
-narrateur|Nino souffle comme le vent.
-narrateur|Une fois.
-narrateur|Deux fois.
-narrateur|Il fait une pause.
-narrateur|La chambre redevient calme.
-enfant-m|Je souffle. Je fais une pause.
-maman|Bravo, Nino. C'est calme.
-papa|Tu as soufflé. Tu as fait une pause.
-maman|Tu veux reprendre, tout doucement ?
-enfant-m|Oui. Tout doucement.
-narrateur|Nino reprend un cube bleu.
-narrateur|Il construit tout doucement.
-papa|La tour est petite. Elle tient.</t>
+enfant-f|Oh.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, ça va trop vite.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules montent un peu.
+narrateur|Maman s'accroupit à la même hauteur.
+maman|Tu vois les cubes, Nina ?
+enfant-f|Oui, maman.
+papa|Ta poitrine va vite, Nina ?
+enfant-f|Un peu, papa.
+enfant-f|C'est trop.
+narrateur|Nina souffle vers ses mains.
+enfant-f|Fouu.
+narrateur|Elle fait une pause, près du lit.
+narrateur|L'éclat de lit tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>oiseau,cubes</t>
+          <t>cubes</t>
         </is>
       </c>
     </row>
@@ -1402,17 +1418,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Le corps de Nino va vite. Que fait-il ?</t>
+          <t>Le corps de Nina va vite. Que fait-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps de Nino va vite. Que fait-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le corps de Nina va &lt;emphasis level="moderate"&gt;vite&lt;/emphasis&gt;. Que fait-elle ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le corps de Gaëlle va vite. Que fait-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le corps de Nina va &lt;emphasis&gt;vite&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1475,7 +1491,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1486,7 +1502,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1501,34 +1517,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>vite</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1543,7 +1563,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1553,13 +1573,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_corps_va_vite_que_fait_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Le corps de Nino va vite.
-narrateur|Que fait-il ?</t>
+          <t>narrateur|Le corps de Nina va vite.
+narrateur|Que fait-elle ?</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1606,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino a soufflé. Il a fait une pause. Son corps a ralenti. Tu as entendu l'oiseau ? Oui. Il chante encore. La chambre est calme. On reprend. Un cube glisse encore. Nino sent encore sa poitrine. Je souffle. Je fais une pause. Oui. Souffler. Puis une pause. Tu t'assois. Tu souffles. Nino s'assoit. Il souffle. Une fois. Deux fois. Il fait une pause. Tes mains sont sur tes genoux. Bravo. Tu as repris. La tour est petite. Elle tient. C'est bien.</t>
+          <t>Nina pose un cube sur le bois. Un, maman. Elle pose un autre, plus bas. Tu veux la pile avec moi ? Oui, chacun un cube. Papa ne dit rien, d'abord. Je tiens le mien. Moi aussi. Merci, Nina. Papa a vu les deux, près du lit. Le bois colle un peu, sous les doigts. Il est lisse. Ils essuient le cube du plat de la main. Nina tient son cube, plus bas. Il tient ! Tu le vois, le bleu ? Oui, papa. Au milieu, Nina ? J'y vais. Nina pousse le cube, sans se presser. Papa suit le bois des yeux. La pile danse une fois. Un. Deux. Le ventre de Nina se desserre. Les épaules descendent un peu. On reste près du lit ? Oui. Tes mains sont au chaud ? Un peu, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino a soufflé. Il a fait une pause. Son corps a ralenti. Tu as entendu l'oiseau ? Oui. Il chante encore. La chambre est calme. On reprend. Un cube glisse encore. Nino sent encore sa poitrine. Je souffle. Je fais une pause. Oui. Souffler. Puis une pause. Tu t'assois. Tu souffles. Nino s'assoit. Il souffle. Une fois. Deux fois. Il fait une pause. Tes mains sont sur tes genoux. Bravo. Tu as repris. La tour est petite. Elle tient. C'est bien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina pose un cube sur le bois. Un, maman. Elle pose un autre, plus bas. Tu veux la pile avec moi ? Oui, chacun un cube. Papa ne dit rien, d'abord. Je tiens le mien. Moi aussi. Merci, Nina. Papa a vu les deux, près du lit. Le bois colle un peu, sous les doigts. Il est lisse. Ils essuient le cube du plat de la main. Nina tient son cube, plus bas. Il tient ! Tu le vois, le bleu ? Oui, papa. Au milieu, Nina ? J'y vais. Nina pousse le cube, sans se presser. Papa suit le bois des yeux. La pile danse une fois. Un. Deux. Le ventre de Nina se desserre. Les épaules descendent un peu. On reste près du lit ? Oui. Tes mains sont au chaud ? Un peu, papa.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Gaëlle a soufflé. Elle a fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Son corps a ralenti.&lt;/slow&gt; [pause]</t>
+          <t>Nina pose un cube sur le bois. Un, maman. Elle pose un autre, plus bas. Tu veux la pile avec moi ? Oui, chacun un cube. Papa ne dit rien, d'abord. Je tiens le mien. Moi aussi. Merci, Nina. Papa a vu les deux, près du lit. Le bois colle un peu, sous les doigts. Il est lisse. Ils essuient le cube du plat de la main. Nina tient son cube, plus bas. Il tient ! Tu le vois, le bleu ? Oui, papa. Au milieu, Nina ? J'y vais. Nina pousse le cube, sans se presser. Papa suit le bois des yeux. La pile danse une fois. Un. Deux. Le ventre de Nina se desserre. Les épaules descendent un peu. On reste près du lit ? Oui. Tes mains sont au chaud ? Un peu, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,18 +1663,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1684,23 +1704,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1729,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,35 +1741,45 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_pose_plus_bas_ils_tiennent; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino a soufflé.
-narrateur|Il a fait une pause.
-narrateur|Son corps a ralenti.
-papa|Tu as entendu l'oiseau ?
-enfant-m|Oui. Il chante encore.
-maman|La chambre est calme. On reprend.
-narrateur|Un cube glisse encore.
-narrateur|Nino sent encore sa poitrine.
-enfant-m|Je souffle. Je fais une pause.
-maman|Oui. Souffler. Puis une pause.
-papa|Tu t'assois. Tu souffles.
-narrateur|Nino s'assoit.
-narrateur|Il souffle.
-narrateur|Une fois.
-narrateur|Deux fois.
-narrateur|Il fait une pause.
-maman|Tes mains sont sur tes genoux.
-papa|Bravo. Tu as repris.
-enfant-m|La tour est petite.
-maman|Elle tient. C'est bien.</t>
+          <t>narrateur|Nina pose un cube sur le bois.
+enfant-f|Un, maman.
+narrateur|Elle pose un autre, plus bas.
+papa|Tu veux la pile avec moi ?
+enfant-f|Oui, chacun un cube.
+narrateur|Papa ne dit rien, d'abord.
+papa|Je tiens le mien.
+enfant-f|Moi aussi.
+papa|Merci, Nina.
+narrateur|Papa a vu les deux, près du lit.
+maman|Le bois colle un peu, sous les doigts.
+enfant-f|Il est lisse.
+narrateur|Ils essuient le cube du plat de la main.
+narrateur|Nina tient son cube, plus bas.
+enfant-f|Il tient !
+papa|Tu le vois, le bleu ?
+enfant-f|Oui, papa.
+maman|Au milieu, Nina ?
+enfant-f|J'y vais.
+narrateur|Nina pousse le cube, sans se presser.
+narrateur|Papa suit le bois des yeux.
+narrateur|La pile danse une fois.
+enfant-f|Un.
+papa|Deux.
+narrateur|Le ventre de Nina se desserre.
+narrateur|Les épaules descendent un peu.
+maman|On reste près du lit ?
+enfant-f|Oui.
+papa|Tes mains sont au chaud ?
+enfant-f|Un peu, papa.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1781,17 +1811,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino pose un cube bleu. Le doudou regarde depuis le lit. Elle tient, maman. Oui. Tu as fini ta petite tour ? Oui. On range un cube ensemble ? Un cube. Puis le doudou. Nino range un cube. Il prend le doudou. Le doudou est doux, hein ? Oui. Il est chaud. Le rideau jaune bouge encore. La chambre est calme.</t>
+          <t>Maman pousse les cubes vers le lit. La pile est un peu haute. Les cubes, maintenant ! Nina avance trop, tout de suite. Elle monte les cubes sur le lit. Plus haut ! Le coton est mou, sous les cubes. Ils partent ! Les cubes glissent vers le bord. Nina avance les mains, trop vite. La pile s'effondre sur le coton. Oh. Nina refuse d'empiler, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le lit, un instant. Elle écoute le bois du lit. Sur le bois, un éclat de lit luit. Là, sur le bois. Nina souffle vers le bois. Fouu. Elle fait une pause, sur le bois. Tu tends le cube, papa ? Papa ne dit rien. Il souffle, puis tend le cube. Oui. On arrête la pile ? Oui, maman. Le bois sent le coton tiède. Les cubes sont là, un peu au bord. Nina les pose près de papa. Papa les rend, sans presser. Clic. Clic. Le cube est bien posé ? Oui, maman. Le bois est lisse, Nina ? Un peu. Ils se passent un cube, près d'eux. Le bois est lisse, sous les genoux. C'est plus facile. Le rayon est calme ? Oui, maman. Un rayon passe sur le bois. Il allume le point.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino pose un cube bleu. Le doudou regarde depuis le lit. Elle tient, maman. Oui. Tu as fini ta petite tour ? Oui. On range un cube ensemble ? Un cube. Puis le doudou. Nino range un cube. Il prend le doudou. Le doudou est doux, hein ? Oui. Il est chaud. Le rideau jaune bouge encore. La chambre est calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pousse les cubes vers le lit. La pile est un peu haute. Les cubes, maintenant ! Nina avance trop, tout de suite. Elle monte les cubes sur le lit. Plus haut ! Le coton est mou, sous les cubes. Ils partent ! Les cubes glissent vers le bord. Nina avance les mains, trop vite. La pile s'effondre sur le coton. Oh. Nina refuse d'empiler, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le lit, un instant. Elle écoute le bois du lit. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de lit&lt;/emphasis&gt; luit. Là, sur le bois. Nina souffle vers le bois. Fouu. Elle fait une pause, sur le bois. Tu tends le cube, papa ? Papa ne dit rien. Il souffle, puis tend le cube. Oui. On arrête la pile ? Oui, maman. Le bois sent le coton tiède. Les cubes sont là, un peu au bord. Nina les pose près de papa. Papa les rend, sans presser. Clic. Clic. Le cube est bien posé ? Oui, maman. Le bois est lisse, Nina ? Un peu. Ils se passent un cube, près d'eux. Le bois est lisse, sous les genoux. C'est plus facile. Le rayon est calme ? Oui, maman. Un rayon passe sur le bois. Il allume le point.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Gaëlle pose un cube bleu. Maman reste sur le tapis.&lt;/slow&gt; [pause]</t>
+          <t>Maman pousse les cubes vers le lit. La pile est un peu haute. Les cubes, maintenant ! Nina avance trop, tout de suite. Elle monte les cubes sur le lit. Plus haut ! Le coton est mou, sous les cubes. Ils partent ! Les cubes glissent vers le bord. Nina avance les mains, trop vite. La pile s'effondre sur le coton. Oh. Nina refuse d'empiler, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le lit, un instant. Elle écoute le bois du lit. Sur le bois, un &lt;emphasis&gt;éclat de lit&lt;/emphasis&gt; luit. Là, sur le bois. Nina souffle vers le bois. Fouu. Elle fait une pause, sur le bois. Tu tends le cube, papa ? Papa ne dit rien. Il souffle, puis tend le cube. Oui. On arrête la pile ? Oui, maman. Le bois sent le coton tiède. Les cubes sont là, un peu au bord. Nina les pose près de papa. Papa les rend, sans presser. Clic. Clic. Le cube est bien posé ? Oui, maman. Le bois est lisse, Nina ? Un peu. Ils se passent un cube, près d'eux. Le bois est lisse, sous les genoux. C'est plus facile. Le rayon est calme ? Oui, maman. Un rayon passe sur le bois. Il allume le point. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,18 +1868,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1870,28 +1900,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de lit</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,10 +1934,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1912,24 +1946,65 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=les_cubes_glissent_sur_le_coton; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino pose un cube bleu.
-narrateur|Le doudou regarde depuis le lit.
-enfant-m|Elle tient, maman.
-maman|Oui. Tu as fini ta petite tour ?
-enfant-m|Oui.
-maman|On range un cube ensemble ?
-enfant-m|Un cube. Puis le doudou.
-narrateur|Nino range un cube.
-narrateur|Il prend le doudou.
-papa|Le doudou est doux, hein ?
-enfant-m|Oui. Il est chaud.
-narrateur|Le rideau jaune bouge encore.
-narrateur|La chambre est calme.</t>
+          <t>narrateur|Maman pousse les cubes vers le lit.
+narrateur|La pile est un peu haute.
+enfant-f|Les cubes, maintenant !
+narrateur|Nina avance trop, tout de suite.
+narrateur|Elle monte les cubes sur le lit.
+enfant-f|Plus haut !
+narrateur|Le coton est mou, sous les cubes.
+enfant-f|Ils partent !
+narrateur|Les cubes glissent vers le bord.
+narrateur|Nina avance les mains, trop vite.
+narrateur|La pile s'effondre sur le coton.
+enfant-f|Oh.
+narrateur|Nina refuse d'empiler, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le lit, un instant.
+narrateur|Elle écoute le bois du lit.
+narrateur|Sur le bois, un éclat de lit luit.
+enfant-f|Là, sur le bois.
+narrateur|Nina souffle vers le bois.
+enfant-f|Fouu.
+narrateur|Elle fait une pause, sur le bois.
+enfant-f|Tu tends le cube, papa ?
+narrateur|Papa ne dit rien.
+narrateur|Il souffle, puis tend le cube.
+papa|Oui.
+maman|On arrête la pile ?
+enfant-f|Oui, maman.
+narrateur|Le bois sent le coton tiède.
+narrateur|Les cubes sont là, un peu au bord.
+narrateur|Nina les pose près de papa.
+narrateur|Papa les rend, sans presser.
+enfant-f|Clic.
+papa|Clic.
+maman|Le cube est bien posé ?
+enfant-f|Oui, maman.
+papa|Le bois est lisse, Nina ?
+enfant-f|Un peu.
+narrateur|Ils se passent un cube, près d'eux.
+narrateur|Le bois est lisse, sous les genoux.
+enfant-f|C'est plus facile.
+maman|Le rayon est calme ?
+enfant-f|Oui, maman.
+papa|Un rayon passe sur le bois.
+enfant-f|Il allume le point.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>cubes</t>
         </is>
       </c>
     </row>
@@ -1956,17 +2031,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Nino. Ta tour est petite. Elle tient.</t>
+          <t>Ils restent près du lit. Maman lisse un coin de coton. Les cubes ont glissé, papa. Tu l'as vu, toi ? Oui, près du lit. On est bien, ici. Nina tapote le bois du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. Le lit est resté, Nina. Oui, avec les cubes. Les cubes sont restés. Ça sent le coton, un peu tiède. Et le bois, papa. Oui, dans l'air. Le lit reste sous le rayon. Un éclat de lit tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Nino. Ta tour est petite. Elle tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du lit. Maman lisse un coin de coton. Les cubes ont glissé, papa. Tu l'as vu, toi ? Oui, près du lit. On est bien, ici. Nina tapote le bois du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. Le lit est resté, Nina. Oui, avec les cubes. Les cubes sont restés. Ça sent le coton, un peu tiède. Et le bois, papa. Oui, dans l'air. Le lit reste sous le rayon. Un &lt;emphasis level="moderate"&gt;éclat de lit&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du lit. Maman lisse un coin de coton. Les cubes ont glissé, papa. Tu l'as vu, toi ? Oui, près du lit. On est bien, ici. Nina tapote le bois du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. Le lit est resté, Nina. Oui, avec les cubes. Les cubes sont restés. Ça sent le coton, un peu tiède. Et le bois, papa. Oui, dans l'air. Le lit reste sous le rayon. Un &lt;emphasis&gt;éclat de lit&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2013,7 +2088,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2096,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2033,12 +2108,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2047,14 +2122,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de lit</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2066,11 +2145,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2079,26 +2158,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai soufflé. J'ai fait une pause.
-maman|Bravo, Nino.
-papa|Ta tour est petite. Elle tient.</t>
+          <t>narrateur|Ils restent près du lit.
+narrateur|Maman lisse un coin de coton.
+enfant-f|Les cubes ont glissé, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui, près du lit.
+maman|On est bien, ici.
+narrateur|Nina tapote le bois du doigt.
+enfant-f|Il a une trace de doigt.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le lit est resté, Nina.
+enfant-f|Oui, avec les cubes.
+maman|Les cubes sont restés.
+narrateur|Ça sent le coton, un peu tiède.
+enfant-f|Et le bois, papa.
+papa|Oui, dans l'air.
+narrateur|Le lit reste sous le rayon.
+narrateur|Un éclat de lit tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2183,6 +2281,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>